<commit_message>
Deployed 9c2e951 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/artifacts/Liu2024_PM25_CFTR_SOMA.xlsx
+++ b/artifacts/Liu2024_PM25_CFTR_SOMA.xlsx
@@ -757,7 +757,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>fold change (UO:0000193)</t>
+          <t>UO:0000193</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr"/>
@@ -789,7 +789,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>fold change (UO:0000193)</t>
+          <t>UO:0000193</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr"/>
@@ -823,7 +823,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>fold change (UO:0000193)</t>
+          <t>UO:0000193</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -855,7 +855,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>fold change (UO:0000193)</t>
+          <t>UO:0000193</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -889,7 +889,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>percent (UO:0000187)</t>
+          <t>UO:0000187</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>percent (UO:0000187)</t>
+          <t>UO:0000187</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr"/>
@@ -1221,7 +1221,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>percent (UO:0000187)</t>
+          <t>UO:0000187</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr"/>
@@ -1434,7 +1434,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>fold change vs OVA (UO:0000193)</t>
+          <t>UO:0000193</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -1676,7 +1676,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>fold change vs control (UO:0000193)</t>
+          <t>UO:0000193</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -1704,7 +1704,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>fold change vs control (UO:0000193)</t>
+          <t>UO:0000193</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -2087,7 +2087,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>ug/mL (UO:0000064)</t>
+          <t>UO:0000064</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -2097,7 +2097,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>hour (UO:0000032)</t>
+          <t>UO:0000032</t>
         </is>
       </c>
     </row>
@@ -2129,7 +2129,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>ug/mL (UO:0000064)</t>
+          <t>UO:0000064</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -2139,7 +2139,7 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>hour (UO:0000032)</t>
+          <t>UO:0000032</t>
         </is>
       </c>
     </row>
@@ -2171,7 +2171,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>ug/mL (UO:0000064)</t>
+          <t>UO:0000064</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -2181,7 +2181,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>day (UO:0000033)</t>
+          <t>UO:0000033</t>
         </is>
       </c>
     </row>
@@ -2213,7 +2213,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>mg/kg (UO:0000308)</t>
+          <t>UO:0000308</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -2223,7 +2223,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>day (UO:0000033)</t>
+          <t>UO:0000033</t>
         </is>
       </c>
     </row>
@@ -2255,7 +2255,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>mg/kg (UO:0000308)</t>
+          <t>UO:0000308</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -2265,7 +2265,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>day (UO:0000033)</t>
+          <t>UO:0000033</t>
         </is>
       </c>
     </row>
@@ -2771,7 +2771,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>week (UO:0000034)</t>
+          <t>UO:0000034</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -2830,7 +2830,7 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>week (UO:0000034)</t>
+          <t>UO:0000034</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -2897,7 +2897,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>week (UO:0000034)</t>
+          <t>UO:0000034</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -2960,7 +2960,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>week (UO:0000034)</t>
+          <t>UO:0000034</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -3346,7 +3346,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>fold change (UO:0000193)</t>
+          <t>UO:0000193</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr"/>
@@ -3378,7 +3378,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>fold change (UO:0000193)</t>
+          <t>UO:0000193</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr"/>
@@ -3410,7 +3410,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>fold change (UO:0000193)</t>
+          <t>UO:0000193</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr"/>
@@ -3442,7 +3442,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>fold change (UO:0000193)</t>
+          <t>UO:0000193</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr"/>

</xml_diff>